<commit_message>
Launch evidence-backed request-only beta
</commit_message>
<xml_diff>
--- a/docs/examples/sample-invoice-output.xlsx
+++ b/docs/examples/sample-invoice-output.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Table 1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30,12 +31,17 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2F0D9"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -50,8 +56,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -418,68 +426,110 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>table</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>location</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>rows</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>columns</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>looks_clean</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>has_merged_cells</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>warnings</t>
+          <t>decision</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>accepted</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>1</v>
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>profile</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>page 1</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>4</v>
-      </c>
-      <c r="D2" t="n">
+          <t>invoice-lines-v1</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>profile_version</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1.0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>document_sha256</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>4c6332535cb6b99efdc03cea0f548461622201ad5f3e5c9c6605e83f95914566</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>extraction_fingerprint</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>bfccb01adf74aa2d9d2b46852a5d617cbb0237f9d8951a968e76cfdf3f198ec3</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>records</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
         <v>3</v>
       </c>
-      <c r="E2" t="b">
-        <v>1</v>
-      </c>
-      <c r="F2" t="b">
-        <v>0</v>
-      </c>
-      <c r="G2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>issues</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>severity</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>message</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>source</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -492,117 +542,510 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>source</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>/root/pdf-mcp/docs/examples/sample-invoice.pdf</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="n"/>
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>unit_price</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>issues</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>location</t>
-        </is>
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Widget</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>12.50</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Gadget</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>40.00</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>accepted</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Bolt</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>record</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t>raw</t>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>page</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>table</t>
+        </is>
+      </c>
+      <c r="G1" s="3" t="inlineStr">
+        <is>
+          <t>row</t>
+        </is>
+      </c>
+      <c r="H1" s="3" t="inlineStr">
+        <is>
+          <t>column</t>
+        </is>
+      </c>
+      <c r="I1" s="3" t="inlineStr">
+        <is>
+          <t>bbox</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>page 1</t>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Widget</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Widget</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>[242.948, 136.0, 287.748, 154.0]</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>looks_clean</t>
-        </is>
-      </c>
-      <c r="B3" t="b">
-        <v>1</v>
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>[287.748, 136.0, 315.308, 154.0]</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>warnings</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>unit_price</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>12.50</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>12.50</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>[315.308, 136.0, 352.328, 154.0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>item</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Gadget</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Gadget</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>[242.948, 154.0, 287.748, 172.0]</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Item</t>
-        </is>
+      <c r="A6" t="n">
+        <v>2</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Qty</t>
+          <t>quantity</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Price</t>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>[287.748, 154.0, 315.308, 172.0]</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Widget</t>
-        </is>
+      <c r="A7" t="n">
+        <v>2</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>unit_price</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>12.50</t>
+          <t>40.00</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>40.00</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>[315.308, 154.0, 352.328, 172.0]</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Gadget</t>
-        </is>
+      <c r="A8" t="n">
+        <v>3</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>item</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>40.00</t>
+          <t>Bolt</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Bolt</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" t="n">
+        <v>3</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>[242.948, 172.0, 287.748, 190.0]</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Bolt</t>
-        </is>
+      <c r="A9" t="n">
+        <v>3</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>10</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>3</v>
+      </c>
+      <c r="H9" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>[287.748, 172.0, 315.308, 190.0]</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>unit_price</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
         <is>
           <t>0.25</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>0.25</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>3</v>
+      </c>
+      <c r="H10" t="n">
+        <v>2</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>[315.308, 172.0, 352.328, 190.0]</t>
         </is>
       </c>
     </row>

</xml_diff>